<commit_message>
Add new tools for prefab searching and image replacement, update prefab and character metadata
</commit_message>
<xml_diff>
--- a/Assets/ArtRes/Excel/Character1.xlsx
+++ b/Assets/ArtRes/Excel/Character1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ARPG\Assets\ArtRes\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9051A2B6-C896-494D-9FA5-7C4084585308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1D8D80-8F26-42C4-B7DD-17AD7E5340DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Weapon" sheetId="1" r:id="rId1"/>
@@ -448,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
@@ -490,54 +490,54 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2">
-        <v>15.5</v>
-      </c>
-      <c r="D4" s="2">
-        <v>200</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>200</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B6" s="2">
         <v>2</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C6" s="2">
         <v>18</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D6" s="2">
         <v>300</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="7" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B7" s="2">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C7" s="2">
         <v>22.5</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D7" s="2">
         <v>400</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -588,10 +588,10 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>

</xml_diff>